<commit_message>
feat: add definedName for profile version
Signed-off-by: Mats Johansson <extern.mats.johansson@digg.se>
</commit_message>
<xml_diff>
--- a/document/Avstaemning_REST_API_profil_v_1_2_0_0.xlsx
+++ b/document/Avstaemning_REST_API_profil_v_1_2_0_0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MatsJohansson\repos\rest-api-profil-lint-processor\document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\mats\repos\rest-api-profil-lint-processor\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55DD905-FDA6-4632-BA42-4EC4B8D06E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDDF6FE-C383-4109-8581-5D6A405BA8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="692" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kravlista REST API profil'!$A$1:$F$1</definedName>
+    <definedName name="profilversion">"1.2.0"</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -6961,13 +6965,13 @@
     </xf>
   </cellXfs>
   <cellStyles count="7">
-    <cellStyle name="Bad" xfId="3" builtinId="27"/>
-    <cellStyle name="Good" xfId="2" builtinId="26"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Anteckning" xfId="6" builtinId="10"/>
+    <cellStyle name="Bra" xfId="2" builtinId="26"/>
+    <cellStyle name="Dålig" xfId="3" builtinId="27"/>
+    <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="6" builtinId="10"/>
-    <cellStyle name="Percent" xfId="5" builtinId="5"/>
+    <cellStyle name="Procent" xfId="5" builtinId="5"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
@@ -7332,15 +7336,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AW49"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="21" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="21" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="13" width="10.7109375" style="14" customWidth="1"/>
-    <col min="14" max="23" width="8.7109375" style="14" customWidth="1"/>
-    <col min="24" max="49" width="8.7109375" style="14" hidden="1"/>
-    <col min="50" max="16384" width="9.140625" hidden="1"/>
+    <col min="1" max="13" width="10.68359375" style="14" customWidth="1"/>
+    <col min="14" max="23" width="8.68359375" style="14" customWidth="1"/>
+    <col min="24" max="49" width="8.68359375" style="14" hidden="1" customWidth="1"/>
+    <col min="50" max="16384" width="9.15625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="30" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" s="30" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A1" s="72" t="s">
         <v>130</v>
       </c>
@@ -7367,7 +7371,7 @@
       <c r="V1" s="72"/>
       <c r="W1" s="72"/>
     </row>
-    <row r="2" spans="1:23" ht="155.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="155.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="73" t="s">
         <v>370</v>
       </c>
@@ -7394,7 +7398,7 @@
       <c r="T2" s="75"/>
       <c r="U2" s="76"/>
     </row>
-    <row r="3" spans="1:23" s="32" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" s="32" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="36" t="s">
         <v>197</v>
       </c>
@@ -7404,12 +7408,12 @@
       <c r="E3" s="31"/>
       <c r="F3" s="31"/>
     </row>
-    <row r="4" spans="1:23" s="13" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" s="13" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="13" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="18" t="s">
         <v>134</v>
       </c>
@@ -7426,7 +7430,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="21">
         <f>COUNTIF('Kravlista REST API profil'!E2:E190,"-")</f>
         <v>151</v>
@@ -7451,7 +7455,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="22">
         <f>(A6/SUM(A6:E6))</f>
         <v>1</v>
@@ -7476,13 +7480,13 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:23" s="13" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="9" spans="1:23" s="13" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="13" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="10" spans="1:23" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="37" t="str">
         <f>('Kravlista REST API profil'!$A2)</f>
         <v>Dokumentation</v>
@@ -7492,7 +7496,7 @@
         <v>Datum- och tidsformat</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -7534,7 +7538,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E2:E26,"-")</f>
         <v>23</v>
@@ -7582,7 +7586,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="22">
         <f>(A12/SUM(A12:E12))</f>
         <v>1</v>
@@ -7630,8 +7634,8 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:23" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="15" spans="1:23" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="37" t="str">
         <f>('Kravlista REST API profil'!$A33)</f>
         <v>Resurser</v>
@@ -7641,7 +7645,7 @@
         <v>URL format och namngivning</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -7683,7 +7687,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E33:E40,"-")</f>
         <v>6</v>
@@ -7731,7 +7735,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="22">
         <f>(A17/SUM(A17:E17))</f>
         <v>1</v>
@@ -7779,8 +7783,8 @@
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="20" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="str">
         <f>('Kravlista REST API profil'!$A52)</f>
         <v>Mognad</v>
@@ -7790,7 +7794,7 @@
         <v>Säkerhet</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -7832,7 +7836,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E52:E54,"-")</f>
         <v>3</v>
@@ -7880,7 +7884,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="22">
         <f>(A22/SUM(A22:E22))</f>
         <v>1</v>
@@ -7928,8 +7932,8 @@
         <v>136</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="25" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="37" t="str">
         <f>('Kravlista REST API profil'!$A97)</f>
         <v>API Message</v>
@@ -7939,7 +7943,7 @@
         <v>API Request</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -7981,7 +7985,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E97:E104,"-")</f>
         <v>6</v>
@@ -8029,7 +8033,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="22">
         <f>(A27/SUM(A27:E27))</f>
         <v>1</v>
@@ -8077,8 +8081,8 @@
         <v>136</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="30" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="37" t="str">
         <f>('Kravlista REST API profil'!$A112)</f>
         <v>API Response</v>
@@ -8088,7 +8092,7 @@
         <v>Felhantering</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -8130,7 +8134,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E112:E115,"-")</f>
         <v>3</v>
@@ -8178,7 +8182,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="22">
         <f>(A32/SUM(A32:E32))</f>
         <v>1</v>
@@ -8226,8 +8230,8 @@
         <v>136</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="35" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="37" t="str">
         <f>('Kravlista REST API profil'!$A118)</f>
         <v>Versionshantering</v>
@@ -8237,7 +8241,7 @@
         <v>Webhooks</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -8279,7 +8283,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E118:E142,"-")</f>
         <v>19</v>
@@ -8327,7 +8331,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="22">
         <f>(A37/SUM(A37:E37))</f>
         <v>1</v>
@@ -8375,8 +8379,8 @@
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="40" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="37" t="str">
         <f>('Kravlista REST API profil'!$A149)</f>
         <v>Hypermedia</v>
@@ -8386,7 +8390,7 @@
         <v>Filtrering, namnsättning och sökparametrar</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -8428,7 +8432,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E149:E173,"-")</f>
         <v>19</v>
@@ -8476,7 +8480,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="22">
         <f>(A42/SUM(A42:E42))</f>
         <v>1</v>
@@ -8524,14 +8528,14 @@
         <v>136</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
+    <row r="45" spans="1:13" s="37" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="37" t="str">
         <f>('Kravlista REST API profil'!$A190)</f>
         <v>Cachning</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="18" t="str">
         <f>$A$5</f>
         <v>-</v>
@@ -8553,7 +8557,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="35">
         <f>COUNTIF('Kravlista REST API profil'!E190:E190,"-")</f>
         <v>1</v>
@@ -8583,7 +8587,7 @@
       <c r="K47" s="35"/>
       <c r="L47" s="35"/>
     </row>
-    <row r="48" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="22">
         <f>(A47/SUM(A47:E47))</f>
         <v>1</v>
@@ -8614,7 +8618,7 @@
       <c r="L48" s="23"/>
       <c r="M48" s="24"/>
     </row>
-    <row r="49" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="21" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:W1"/>
@@ -8629,20 +8633,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BJ418"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15.75" zeroHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15.6" zeroHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="18.140625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="92.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.15625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="9.26171875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="92.41796875" style="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="38.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" style="10" customWidth="1"/>
-    <col min="8" max="62" width="0" style="10" hidden="1"/>
-    <col min="63" max="16384" width="8.7109375" style="1" hidden="1"/>
+    <col min="5" max="5" width="11.15625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="38.578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.68359375" style="10" customWidth="1"/>
+    <col min="8" max="62" width="0" style="10" hidden="1" customWidth="1"/>
+    <col min="63" max="16384" width="8.68359375" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:62" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
@@ -8718,7 +8722,7 @@
       <c r="BI1" s="10"/>
       <c r="BJ1" s="10"/>
     </row>
-    <row r="2" spans="1:62" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:62" ht="31.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="53" t="s">
         <v>4</v>
       </c>
@@ -8737,7 +8741,7 @@
       <c r="F2" s="4"/>
       <c r="G2" s="12"/>
     </row>
-    <row r="3" spans="1:62" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:62" ht="31.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="55"/>
       <c r="B3" s="3" t="s">
         <v>200</v>
@@ -8754,7 +8758,7 @@
       <c r="F3" s="4"/>
       <c r="G3" s="12"/>
     </row>
-    <row r="4" spans="1:62" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:62" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="55"/>
       <c r="B4" s="33" t="s">
         <v>5</v>
@@ -8765,7 +8769,7 @@
       <c r="F4" s="42"/>
       <c r="G4" s="12"/>
     </row>
-    <row r="5" spans="1:62" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:62" ht="109.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="55"/>
       <c r="B5" s="3" t="s">
         <v>221</v>
@@ -8782,7 +8786,7 @@
       <c r="F5" s="4"/>
       <c r="G5" s="12"/>
     </row>
-    <row r="6" spans="1:62" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:62" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="55"/>
       <c r="B6" s="3" t="s">
         <v>201</v>
@@ -8799,7 +8803,7 @@
       <c r="F6" s="4"/>
       <c r="G6" s="12"/>
     </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="55"/>
       <c r="B7" s="3" t="s">
         <v>202</v>
@@ -8816,7 +8820,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="12"/>
     </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="55"/>
       <c r="B8" s="3" t="s">
         <v>203</v>
@@ -8833,7 +8837,7 @@
       <c r="F8" s="4"/>
       <c r="G8" s="12"/>
     </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="55"/>
       <c r="B9" s="3" t="s">
         <v>204</v>
@@ -8850,7 +8854,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="12"/>
     </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="55"/>
       <c r="B10" s="3" t="s">
         <v>205</v>
@@ -8867,7 +8871,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="12"/>
     </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="55"/>
       <c r="B11" s="3" t="s">
         <v>206</v>
@@ -8884,7 +8888,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="12"/>
     </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="55"/>
       <c r="B12" s="3" t="s">
         <v>207</v>
@@ -8901,7 +8905,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="12"/>
     </row>
-    <row r="13" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="55"/>
       <c r="B13" s="3" t="s">
         <v>208</v>
@@ -8918,7 +8922,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="12"/>
     </row>
-    <row r="14" spans="1:62" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:62" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="55"/>
       <c r="B14" s="3" t="s">
         <v>209</v>
@@ -8935,7 +8939,7 @@
       <c r="F14" s="4"/>
       <c r="G14" s="12"/>
     </row>
-    <row r="15" spans="1:62" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:62" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="55"/>
       <c r="B15" s="3" t="s">
         <v>210</v>
@@ -8952,7 +8956,7 @@
       <c r="F15" s="4"/>
       <c r="G15" s="12"/>
     </row>
-    <row r="16" spans="1:62" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:62" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="55"/>
       <c r="B16" s="3" t="s">
         <v>211</v>
@@ -8969,7 +8973,7 @@
       <c r="F16" s="4"/>
       <c r="G16" s="12"/>
     </row>
-    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="55"/>
       <c r="B17" s="33" t="s">
         <v>6</v>
@@ -8980,7 +8984,7 @@
       <c r="F17" s="42"/>
       <c r="G17" s="12"/>
     </row>
-    <row r="18" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="55"/>
       <c r="B18" s="3" t="s">
         <v>212</v>
@@ -8997,7 +9001,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="12"/>
     </row>
-    <row r="19" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="55"/>
       <c r="B19" s="3" t="s">
         <v>213</v>
@@ -9014,7 +9018,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="12"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="55"/>
       <c r="B20" s="3" t="s">
         <v>214</v>
@@ -9031,7 +9035,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="12"/>
     </row>
-    <row r="21" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="55"/>
       <c r="B21" s="3" t="s">
         <v>215</v>
@@ -9048,7 +9052,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="12"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="55"/>
       <c r="B22" s="3" t="s">
         <v>216</v>
@@ -9065,7 +9069,7 @@
       <c r="F22" s="4"/>
       <c r="G22" s="12"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="55"/>
       <c r="B23" s="3" t="s">
         <v>217</v>
@@ -9082,7 +9086,7 @@
       <c r="F23" s="4"/>
       <c r="G23" s="12"/>
     </row>
-    <row r="24" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="55"/>
       <c r="B24" s="3" t="s">
         <v>218</v>
@@ -9099,7 +9103,7 @@
       <c r="F24" s="4"/>
       <c r="G24" s="12"/>
     </row>
-    <row r="25" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="55"/>
       <c r="B25" s="3" t="s">
         <v>219</v>
@@ -9116,7 +9120,7 @@
       <c r="F25" s="4"/>
       <c r="G25" s="12"/>
     </row>
-    <row r="26" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A26" s="56"/>
       <c r="B26" s="43" t="s">
         <v>220</v>
@@ -9133,7 +9137,7 @@
       <c r="F26" s="44"/>
       <c r="G26" s="12"/>
     </row>
-    <row r="27" spans="1:7" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="78" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="54" t="s">
         <v>7</v>
       </c>
@@ -9152,7 +9156,7 @@
       <c r="F27" s="38"/>
       <c r="G27" s="12"/>
     </row>
-    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="59"/>
       <c r="B28" s="34" t="s">
         <v>118</v>
@@ -9163,7 +9167,7 @@
       <c r="F28" s="42"/>
       <c r="G28" s="12"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="59"/>
       <c r="B29" s="57" t="s">
         <v>223</v>
@@ -9180,7 +9184,7 @@
       <c r="F29" s="4"/>
       <c r="G29" s="12"/>
     </row>
-    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="59"/>
       <c r="B30" s="34" t="s">
         <v>119</v>
@@ -9191,7 +9195,7 @@
       <c r="F30" s="42"/>
       <c r="G30" s="12"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="59"/>
       <c r="B31" s="57" t="s">
         <v>224</v>
@@ -9208,7 +9212,7 @@
       <c r="F31" s="4"/>
       <c r="G31" s="12"/>
     </row>
-    <row r="32" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A32" s="60"/>
       <c r="B32" s="58" t="s">
         <v>225</v>
@@ -9225,7 +9229,7 @@
       <c r="F32" s="44"/>
       <c r="G32" s="12"/>
     </row>
-    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="55" t="s">
         <v>8</v>
       </c>
@@ -9238,7 +9242,7 @@
       <c r="F33" s="48"/>
       <c r="G33" s="12"/>
     </row>
-    <row r="34" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="55"/>
       <c r="B34" s="3" t="s">
         <v>226</v>
@@ -9255,7 +9259,7 @@
       <c r="F34" s="4"/>
       <c r="G34" s="12"/>
     </row>
-    <row r="35" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="55"/>
       <c r="B35" s="3" t="s">
         <v>227</v>
@@ -9272,7 +9276,7 @@
       <c r="F35" s="4"/>
       <c r="G35" s="12"/>
     </row>
-    <row r="36" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="55"/>
       <c r="B36" s="3" t="s">
         <v>228</v>
@@ -9289,7 +9293,7 @@
       <c r="F36" s="4"/>
       <c r="G36" s="12"/>
     </row>
-    <row r="37" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="55"/>
       <c r="B37" s="3" t="s">
         <v>229</v>
@@ -9306,7 +9310,7 @@
       <c r="F37" s="4"/>
       <c r="G37" s="12"/>
     </row>
-    <row r="38" spans="1:7" ht="167.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="167.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="55"/>
       <c r="B38" s="3" t="s">
         <v>230</v>
@@ -9323,7 +9327,7 @@
       <c r="F38" s="4"/>
       <c r="G38" s="12"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="55"/>
       <c r="B39" s="33" t="s">
         <v>121</v>
@@ -9334,7 +9338,7 @@
       <c r="F39" s="42"/>
       <c r="G39" s="12"/>
     </row>
-    <row r="40" spans="1:7" ht="96" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="96" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A40" s="56"/>
       <c r="B40" s="43" t="s">
         <v>231</v>
@@ -9351,7 +9355,7 @@
       <c r="F40" s="44"/>
       <c r="G40" s="12"/>
     </row>
-    <row r="41" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="59" t="s">
         <v>9</v>
       </c>
@@ -9364,7 +9368,7 @@
       <c r="F41" s="48"/>
       <c r="G41" s="12"/>
     </row>
-    <row r="42" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="59"/>
       <c r="B42" s="57" t="s">
         <v>232</v>
@@ -9381,7 +9385,7 @@
       <c r="F42" s="4"/>
       <c r="G42" s="12"/>
     </row>
-    <row r="43" spans="1:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="59"/>
       <c r="B43" s="57" t="s">
         <v>233</v>
@@ -9398,7 +9402,7 @@
       <c r="F43" s="4"/>
       <c r="G43" s="12"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="59"/>
       <c r="B44" s="57" t="s">
         <v>234</v>
@@ -9415,7 +9419,7 @@
       <c r="F44" s="4"/>
       <c r="G44" s="12"/>
     </row>
-    <row r="45" spans="1:7" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="109.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="59"/>
       <c r="B45" s="57" t="s">
         <v>235</v>
@@ -9432,7 +9436,7 @@
       <c r="F45" s="4"/>
       <c r="G45" s="12"/>
     </row>
-    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="59"/>
       <c r="B46" s="34" t="s">
         <v>123</v>
@@ -9443,7 +9447,7 @@
       <c r="F46" s="42"/>
       <c r="G46" s="12"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="59"/>
       <c r="B47" s="57" t="s">
         <v>236</v>
@@ -9460,7 +9464,7 @@
       <c r="F47" s="4"/>
       <c r="G47" s="12"/>
     </row>
-    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="59"/>
       <c r="B48" s="34" t="s">
         <v>124</v>
@@ -9471,7 +9475,7 @@
       <c r="F48" s="42"/>
       <c r="G48" s="12"/>
     </row>
-    <row r="49" spans="1:7" ht="47.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="47.1" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="59"/>
       <c r="B49" s="57" t="s">
         <v>237</v>
@@ -9488,7 +9492,7 @@
       <c r="F49" s="4"/>
       <c r="G49" s="12"/>
     </row>
-    <row r="50" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="59"/>
       <c r="B50" s="57" t="s">
         <v>238</v>
@@ -9505,7 +9509,7 @@
       <c r="F50" s="4"/>
       <c r="G50" s="12"/>
     </row>
-    <row r="51" spans="1:7" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" ht="47.1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A51" s="60"/>
       <c r="B51" s="58" t="s">
         <v>239</v>
@@ -9522,7 +9526,7 @@
       <c r="F51" s="44"/>
       <c r="G51" s="12"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="59" t="s">
         <v>10</v>
       </c>
@@ -9541,7 +9545,7 @@
       <c r="F52" s="39"/>
       <c r="G52" s="12"/>
     </row>
-    <row r="53" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="59"/>
       <c r="B53" s="57" t="s">
         <v>241</v>
@@ -9558,7 +9562,7 @@
       <c r="F53" s="4"/>
       <c r="G53" s="12"/>
     </row>
-    <row r="54" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A54" s="60"/>
       <c r="B54" s="58" t="s">
         <v>242</v>
@@ -9575,7 +9579,7 @@
       <c r="F54" s="44"/>
       <c r="G54" s="12"/>
     </row>
-    <row r="55" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="59" t="s">
         <v>21</v>
       </c>
@@ -9588,7 +9592,7 @@
       <c r="F55" s="48"/>
       <c r="G55" s="12"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="59"/>
       <c r="B56" s="57" t="s">
         <v>337</v>
@@ -9605,7 +9609,7 @@
       <c r="F56" s="4"/>
       <c r="G56" s="12"/>
     </row>
-    <row r="57" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="59"/>
       <c r="B57" s="57" t="s">
         <v>338</v>
@@ -9622,7 +9626,7 @@
       <c r="F57" s="4"/>
       <c r="G57" s="12"/>
     </row>
-    <row r="58" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="59"/>
       <c r="B58" s="57" t="s">
         <v>339</v>
@@ -9639,7 +9643,7 @@
       <c r="F58" s="4"/>
       <c r="G58" s="12"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="59"/>
       <c r="B59" s="57" t="s">
         <v>340</v>
@@ -9656,7 +9660,7 @@
       <c r="F59" s="4"/>
       <c r="G59" s="12"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="59"/>
       <c r="B60" s="57" t="s">
         <v>341</v>
@@ -9673,7 +9677,7 @@
       <c r="F60" s="4"/>
       <c r="G60" s="12"/>
     </row>
-    <row r="61" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="59"/>
       <c r="B61" s="57" t="s">
         <v>342</v>
@@ -9690,7 +9694,7 @@
       <c r="F61" s="4"/>
       <c r="G61" s="12"/>
     </row>
-    <row r="62" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="59"/>
       <c r="B62" s="34" t="s">
         <v>93</v>
@@ -9701,7 +9705,7 @@
       <c r="F62" s="42"/>
       <c r="G62" s="12"/>
     </row>
-    <row r="63" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="59"/>
       <c r="B63" s="57" t="s">
         <v>343</v>
@@ -9718,7 +9722,7 @@
       <c r="F63" s="4"/>
       <c r="G63" s="12"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="59"/>
       <c r="B64" s="57" t="s">
         <v>344</v>
@@ -9735,7 +9739,7 @@
       <c r="F64" s="4"/>
       <c r="G64" s="12"/>
     </row>
-    <row r="65" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="59"/>
       <c r="B65" s="57" t="s">
         <v>345</v>
@@ -9752,7 +9756,7 @@
       <c r="F65" s="4"/>
       <c r="G65" s="12"/>
     </row>
-    <row r="66" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="59"/>
       <c r="B66" s="57" t="s">
         <v>346</v>
@@ -9769,7 +9773,7 @@
       <c r="F66" s="4"/>
       <c r="G66" s="12"/>
     </row>
-    <row r="67" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="59"/>
       <c r="B67" s="57" t="s">
         <v>347</v>
@@ -9786,7 +9790,7 @@
       <c r="F67" s="4"/>
       <c r="G67" s="12"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="59"/>
       <c r="B68" s="57" t="s">
         <v>348</v>
@@ -9803,7 +9807,7 @@
       <c r="F68" s="4"/>
       <c r="G68" s="12"/>
     </row>
-    <row r="69" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="59"/>
       <c r="B69" s="57" t="s">
         <v>349</v>
@@ -9820,7 +9824,7 @@
       <c r="F69" s="4"/>
       <c r="G69" s="12"/>
     </row>
-    <row r="70" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="59"/>
       <c r="B70" s="57" t="s">
         <v>350</v>
@@ -9837,7 +9841,7 @@
       <c r="F70" s="4"/>
       <c r="G70" s="12"/>
     </row>
-    <row r="71" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="59"/>
       <c r="B71" s="57" t="s">
         <v>351</v>
@@ -9854,7 +9858,7 @@
       <c r="F71" s="4"/>
       <c r="G71" s="12"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="59"/>
       <c r="B72" s="34" t="s">
         <v>94</v>
@@ -9865,7 +9869,7 @@
       <c r="F72" s="42"/>
       <c r="G72" s="12"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="59"/>
       <c r="B73" s="57" t="s">
         <v>352</v>
@@ -9882,7 +9886,7 @@
       <c r="F73" s="4"/>
       <c r="G73" s="12"/>
     </row>
-    <row r="74" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="59"/>
       <c r="B74" s="34" t="s">
         <v>95</v>
@@ -9893,7 +9897,7 @@
       <c r="F74" s="42"/>
       <c r="G74" s="12"/>
     </row>
-    <row r="75" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="59"/>
       <c r="B75" s="57" t="s">
         <v>353</v>
@@ -9910,7 +9914,7 @@
       <c r="F75" s="4"/>
       <c r="G75" s="12"/>
     </row>
-    <row r="76" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="59"/>
       <c r="B76" s="57" t="s">
         <v>354</v>
@@ -9927,7 +9931,7 @@
       <c r="F76" s="4"/>
       <c r="G76" s="12"/>
     </row>
-    <row r="77" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="59"/>
       <c r="B77" s="57" t="s">
         <v>355</v>
@@ -9944,7 +9948,7 @@
       <c r="F77" s="4"/>
       <c r="G77" s="12"/>
     </row>
-    <row r="78" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" s="59"/>
       <c r="B78" s="57" t="s">
         <v>356</v>
@@ -9961,7 +9965,7 @@
       <c r="F78" s="4"/>
       <c r="G78" s="12"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" s="59"/>
       <c r="B79" s="57" t="s">
         <v>357</v>
@@ -9978,7 +9982,7 @@
       <c r="F79" s="4"/>
       <c r="G79" s="12"/>
     </row>
-    <row r="80" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" s="59"/>
       <c r="B80" s="34" t="s">
         <v>23</v>
@@ -9989,7 +9993,7 @@
       <c r="F80" s="42"/>
       <c r="G80" s="12"/>
     </row>
-    <row r="81" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" s="59"/>
       <c r="B81" s="57" t="s">
         <v>358</v>
@@ -10006,7 +10010,7 @@
       <c r="F81" s="4"/>
       <c r="G81" s="12"/>
     </row>
-    <row r="82" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" s="59"/>
       <c r="B82" s="57" t="s">
         <v>359</v>
@@ -10023,7 +10027,7 @@
       <c r="F82" s="4"/>
       <c r="G82" s="12"/>
     </row>
-    <row r="83" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" s="59"/>
       <c r="B83" s="57" t="s">
         <v>360</v>
@@ -10040,7 +10044,7 @@
       <c r="F83" s="4"/>
       <c r="G83" s="12"/>
     </row>
-    <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" s="59"/>
       <c r="B84" s="34" t="s">
         <v>96</v>
@@ -10051,7 +10055,7 @@
       <c r="F84" s="42"/>
       <c r="G84" s="12"/>
     </row>
-    <row r="85" spans="1:7" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="35.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" s="59"/>
       <c r="B85" s="57" t="s">
         <v>361</v>
@@ -10068,7 +10072,7 @@
       <c r="F85" s="4"/>
       <c r="G85" s="12"/>
     </row>
-    <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" s="59"/>
       <c r="B86" s="34" t="s">
         <v>97</v>
@@ -10079,7 +10083,7 @@
       <c r="F86" s="42"/>
       <c r="G86" s="12"/>
     </row>
-    <row r="87" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" s="59"/>
       <c r="B87" s="57" t="s">
         <v>362</v>
@@ -10096,7 +10100,7 @@
       <c r="F87" s="4"/>
       <c r="G87" s="12"/>
     </row>
-    <row r="88" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" s="59"/>
       <c r="B88" s="34" t="s">
         <v>98</v>
@@ -10107,7 +10111,7 @@
       <c r="F88" s="42"/>
       <c r="G88" s="12"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" s="59"/>
       <c r="B89" s="57" t="s">
         <v>363</v>
@@ -10124,7 +10128,7 @@
       <c r="F89" s="4"/>
       <c r="G89" s="12"/>
     </row>
-    <row r="90" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" s="59"/>
       <c r="B90" s="34" t="s">
         <v>99</v>
@@ -10135,7 +10139,7 @@
       <c r="F90" s="42"/>
       <c r="G90" s="12"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" s="59"/>
       <c r="B91" s="57" t="s">
         <v>364</v>
@@ -10152,7 +10156,7 @@
       <c r="F91" s="4"/>
       <c r="G91" s="12"/>
     </row>
-    <row r="92" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" s="59"/>
       <c r="B92" s="57" t="s">
         <v>365</v>
@@ -10169,7 +10173,7 @@
       <c r="F92" s="4"/>
       <c r="G92" s="12"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A93" s="59"/>
       <c r="B93" s="57" t="s">
         <v>366</v>
@@ -10186,7 +10190,7 @@
       <c r="F93" s="4"/>
       <c r="G93" s="12"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" s="59"/>
       <c r="B94" s="57" t="s">
         <v>367</v>
@@ -10203,7 +10207,7 @@
       <c r="F94" s="4"/>
       <c r="G94" s="12"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" s="59"/>
       <c r="B95" s="57" t="s">
         <v>368</v>
@@ -10220,7 +10224,7 @@
       <c r="F95" s="4"/>
       <c r="G95" s="12"/>
     </row>
-    <row r="96" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" ht="15.9" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A96" s="60"/>
       <c r="B96" s="58" t="s">
         <v>369</v>
@@ -10237,7 +10241,7 @@
       <c r="F96" s="44"/>
       <c r="G96" s="12"/>
     </row>
-    <row r="97" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" s="59" t="s">
         <v>11</v>
       </c>
@@ -10256,7 +10260,7 @@
       <c r="F97" s="39"/>
       <c r="G97" s="12"/>
     </row>
-    <row r="98" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A98" s="59"/>
       <c r="B98" s="34" t="s">
         <v>100</v>
@@ -10267,7 +10271,7 @@
       <c r="F98" s="42"/>
       <c r="G98" s="12"/>
     </row>
-    <row r="99" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A99" s="59"/>
       <c r="B99" s="57" t="s">
         <v>244</v>
@@ -10284,7 +10288,7 @@
       <c r="F99" s="4"/>
       <c r="G99" s="12"/>
     </row>
-    <row r="100" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A100" s="59"/>
       <c r="B100" s="34" t="s">
         <v>101</v>
@@ -10295,7 +10299,7 @@
       <c r="F100" s="42"/>
       <c r="G100" s="12"/>
     </row>
-    <row r="101" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A101" s="59"/>
       <c r="B101" s="57" t="s">
         <v>245</v>
@@ -10312,7 +10316,7 @@
       <c r="F101" s="4"/>
       <c r="G101" s="12"/>
     </row>
-    <row r="102" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A102" s="59"/>
       <c r="B102" s="57" t="s">
         <v>246</v>
@@ -10329,7 +10333,7 @@
       <c r="F102" s="4"/>
       <c r="G102" s="12"/>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A103" s="59"/>
       <c r="B103" s="57" t="s">
         <v>247</v>
@@ -10346,7 +10350,7 @@
       <c r="F103" s="4"/>
       <c r="G103" s="12"/>
     </row>
-    <row r="104" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:7" ht="15.9" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A104" s="60"/>
       <c r="B104" s="58" t="s">
         <v>319</v>
@@ -10363,7 +10367,7 @@
       <c r="F104" s="44"/>
       <c r="G104" s="12"/>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" s="62" t="s">
         <v>12</v>
       </c>
@@ -10382,7 +10386,7 @@
       <c r="F105" s="39"/>
       <c r="G105" s="12"/>
     </row>
-    <row r="106" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A106" s="59"/>
       <c r="B106" s="34" t="s">
         <v>102</v>
@@ -10393,7 +10397,7 @@
       <c r="F106" s="42"/>
       <c r="G106" s="12"/>
     </row>
-    <row r="107" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A107" s="59"/>
       <c r="B107" s="57" t="s">
         <v>249</v>
@@ -10410,7 +10414,7 @@
       <c r="F107" s="4"/>
       <c r="G107" s="12"/>
     </row>
-    <row r="108" spans="1:7" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" ht="109.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A108" s="59"/>
       <c r="B108" s="57" t="s">
         <v>250</v>
@@ -10427,7 +10431,7 @@
       <c r="F108" s="4"/>
       <c r="G108" s="12"/>
     </row>
-    <row r="109" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A109" s="59"/>
       <c r="B109" s="57" t="s">
         <v>251</v>
@@ -10444,7 +10448,7 @@
       <c r="F109" s="4"/>
       <c r="G109" s="12"/>
     </row>
-    <row r="110" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A110" s="59"/>
       <c r="B110" s="34" t="s">
         <v>103</v>
@@ -10455,7 +10459,7 @@
       <c r="F110" s="42"/>
       <c r="G110" s="12"/>
     </row>
-    <row r="111" spans="1:7" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:7" ht="93.9" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A111" s="60"/>
       <c r="B111" s="58" t="s">
         <v>320</v>
@@ -10472,7 +10476,7 @@
       <c r="F111" s="44"/>
       <c r="G111" s="12"/>
     </row>
-    <row r="112" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A112" s="68" t="s">
         <v>198</v>
       </c>
@@ -10485,7 +10489,7 @@
       <c r="F112" s="65"/>
       <c r="G112" s="12"/>
     </row>
-    <row r="113" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" s="66"/>
       <c r="B113" s="3" t="s">
         <v>321</v>
@@ -10501,7 +10505,7 @@
       </c>
       <c r="F113" s="4"/>
     </row>
-    <row r="114" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A114" s="66"/>
       <c r="B114" s="3" t="s">
         <v>322</v>
@@ -10517,7 +10521,7 @@
       </c>
       <c r="F114" s="4"/>
     </row>
-    <row r="115" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A115" s="67"/>
       <c r="B115" s="50" t="s">
         <v>323</v>
@@ -10534,7 +10538,7 @@
       <c r="F115" s="51"/>
       <c r="G115" s="12"/>
     </row>
-    <row r="116" spans="1:7" ht="126" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="124.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A116" s="79" t="s">
         <v>23</v>
       </c>
@@ -10553,7 +10557,7 @@
       <c r="F116" s="39"/>
       <c r="G116" s="12"/>
     </row>
-    <row r="117" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A117" s="80"/>
       <c r="B117" s="50" t="s">
         <v>335</v>
@@ -10570,7 +10574,7 @@
       <c r="F117" s="51"/>
       <c r="G117" s="12"/>
     </row>
-    <row r="118" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A118" s="59" t="s">
         <v>13</v>
       </c>
@@ -10583,7 +10587,7 @@
       <c r="F118" s="48"/>
       <c r="G118" s="12"/>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A119" s="59"/>
       <c r="B119" s="57" t="s">
         <v>253</v>
@@ -10600,7 +10604,7 @@
       <c r="F119" s="4"/>
       <c r="G119" s="12"/>
     </row>
-    <row r="120" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A120" s="59"/>
       <c r="B120" s="57" t="s">
         <v>254</v>
@@ -10617,7 +10621,7 @@
       <c r="F120" s="4"/>
       <c r="G120" s="12"/>
     </row>
-    <row r="121" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A121" s="59"/>
       <c r="B121" s="57" t="s">
         <v>255</v>
@@ -10634,7 +10638,7 @@
       <c r="F121" s="4"/>
       <c r="G121" s="12"/>
     </row>
-    <row r="122" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" s="59"/>
       <c r="B122" s="34" t="s">
         <v>105</v>
@@ -10645,7 +10649,7 @@
       <c r="F122" s="42"/>
       <c r="G122" s="12"/>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A123" s="59"/>
       <c r="B123" s="57" t="s">
         <v>256</v>
@@ -10662,7 +10666,7 @@
       <c r="F123" s="4"/>
       <c r="G123" s="12"/>
     </row>
-    <row r="124" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A124" s="59"/>
       <c r="B124" s="57" t="s">
         <v>257</v>
@@ -10679,7 +10683,7 @@
       <c r="F124" s="4"/>
       <c r="G124" s="12"/>
     </row>
-    <row r="125" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A125" s="59"/>
       <c r="B125" s="34" t="s">
         <v>106</v>
@@ -10690,7 +10694,7 @@
       <c r="F125" s="42"/>
       <c r="G125" s="12"/>
     </row>
-    <row r="126" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A126" s="59"/>
       <c r="B126" s="57" t="s">
         <v>258</v>
@@ -10707,7 +10711,7 @@
       <c r="F126" s="4"/>
       <c r="G126" s="12"/>
     </row>
-    <row r="127" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" ht="140.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A127" s="59"/>
       <c r="B127" s="57" t="s">
         <v>259</v>
@@ -10724,7 +10728,7 @@
       <c r="F127" s="4"/>
       <c r="G127" s="12"/>
     </row>
-    <row r="128" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A128" s="59"/>
       <c r="B128" s="34" t="s">
         <v>107</v>
@@ -10735,7 +10739,7 @@
       <c r="F128" s="42"/>
       <c r="G128" s="12"/>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A129" s="59"/>
       <c r="B129" s="57" t="s">
         <v>260</v>
@@ -10752,7 +10756,7 @@
       <c r="F129" s="4"/>
       <c r="G129" s="12"/>
     </row>
-    <row r="130" spans="1:7" ht="142.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" ht="142.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A130" s="59"/>
       <c r="B130" s="57" t="s">
         <v>261</v>
@@ -10769,7 +10773,7 @@
       <c r="F130" s="4"/>
       <c r="G130" s="12"/>
     </row>
-    <row r="131" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A131" s="59"/>
       <c r="B131" s="34" t="s">
         <v>108</v>
@@ -10780,7 +10784,7 @@
       <c r="F131" s="42"/>
       <c r="G131" s="12"/>
     </row>
-    <row r="132" spans="1:7" ht="126" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" ht="109.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A132" s="59"/>
       <c r="B132" s="57" t="s">
         <v>262</v>
@@ -10797,7 +10801,7 @@
       <c r="F132" s="4"/>
       <c r="G132" s="12"/>
     </row>
-    <row r="133" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A133" s="59"/>
       <c r="B133" s="34" t="s">
         <v>109</v>
@@ -10808,7 +10812,7 @@
       <c r="F133" s="42"/>
       <c r="G133" s="12"/>
     </row>
-    <row r="134" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A134" s="59"/>
       <c r="B134" s="57" t="s">
         <v>263</v>
@@ -10825,7 +10829,7 @@
       <c r="F134" s="4"/>
       <c r="G134" s="12"/>
     </row>
-    <row r="135" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A135" s="59"/>
       <c r="B135" s="57" t="s">
         <v>264</v>
@@ -10842,7 +10846,7 @@
       <c r="F135" s="4"/>
       <c r="G135" s="12"/>
     </row>
-    <row r="136" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A136" s="59"/>
       <c r="B136" s="57" t="s">
         <v>265</v>
@@ -10859,7 +10863,7 @@
       <c r="F136" s="4"/>
       <c r="G136" s="12"/>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A137" s="59"/>
       <c r="B137" s="57" t="s">
         <v>266</v>
@@ -10876,7 +10880,7 @@
       <c r="F137" s="4"/>
       <c r="G137" s="12"/>
     </row>
-    <row r="138" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A138" s="59"/>
       <c r="B138" s="57" t="s">
         <v>267</v>
@@ -10893,7 +10897,7 @@
       <c r="F138" s="4"/>
       <c r="G138" s="12"/>
     </row>
-    <row r="139" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A139" s="59"/>
       <c r="B139" s="57" t="s">
         <v>268</v>
@@ -10910,7 +10914,7 @@
       <c r="F139" s="4"/>
       <c r="G139" s="12"/>
     </row>
-    <row r="140" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A140" s="59"/>
       <c r="B140" s="57" t="s">
         <v>269</v>
@@ -10927,7 +10931,7 @@
       <c r="F140" s="4"/>
       <c r="G140" s="12"/>
     </row>
-    <row r="141" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A141" s="59"/>
       <c r="B141" s="57" t="s">
         <v>270</v>
@@ -10944,7 +10948,7 @@
       <c r="F141" s="4"/>
       <c r="G141" s="12"/>
     </row>
-    <row r="142" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A142" s="60"/>
       <c r="B142" s="58" t="s">
         <v>271</v>
@@ -10961,7 +10965,7 @@
       <c r="F142" s="44"/>
       <c r="G142" s="12"/>
     </row>
-    <row r="143" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A143" s="77" t="s">
         <v>24</v>
       </c>
@@ -10980,7 +10984,7 @@
       <c r="F143" s="39"/>
       <c r="G143" s="12"/>
     </row>
-    <row r="144" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A144" s="77"/>
       <c r="B144" s="3" t="s">
         <v>273</v>
@@ -10997,7 +11001,7 @@
       <c r="F144" s="4"/>
       <c r="G144" s="12"/>
     </row>
-    <row r="145" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A145" s="77"/>
       <c r="B145" s="3" t="s">
         <v>274</v>
@@ -11014,7 +11018,7 @@
       <c r="F145" s="4"/>
       <c r="G145" s="12"/>
     </row>
-    <row r="146" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A146" s="77"/>
       <c r="B146" s="3" t="s">
         <v>275</v>
@@ -11031,7 +11035,7 @@
       <c r="F146" s="4"/>
       <c r="G146" s="12"/>
     </row>
-    <row r="147" spans="1:7" ht="63" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A147" s="77"/>
       <c r="B147" s="3" t="s">
         <v>276</v>
@@ -11048,7 +11052,7 @@
       <c r="F147" s="4"/>
       <c r="G147" s="12"/>
     </row>
-    <row r="148" spans="1:7" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:7" ht="47.1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A148" s="78"/>
       <c r="B148" s="43" t="s">
         <v>277</v>
@@ -11065,7 +11069,7 @@
       <c r="F148" s="44"/>
       <c r="G148" s="12"/>
     </row>
-    <row r="149" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A149" s="59" t="s">
         <v>14</v>
       </c>
@@ -11084,7 +11088,7 @@
       <c r="F149" s="39"/>
       <c r="G149" s="12"/>
     </row>
-    <row r="150" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A150" s="59"/>
       <c r="B150" s="34" t="s">
         <v>110</v>
@@ -11095,7 +11099,7 @@
       <c r="F150" s="42"/>
       <c r="G150" s="12"/>
     </row>
-    <row r="151" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A151" s="59"/>
       <c r="B151" s="57" t="s">
         <v>279</v>
@@ -11112,7 +11116,7 @@
       <c r="F151" s="4"/>
       <c r="G151" s="12"/>
     </row>
-    <row r="152" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A152" s="59"/>
       <c r="B152" s="57" t="s">
         <v>280</v>
@@ -11129,7 +11133,7 @@
       <c r="F152" s="4"/>
       <c r="G152" s="12"/>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A153" s="59"/>
       <c r="B153" s="57" t="s">
         <v>281</v>
@@ -11146,7 +11150,7 @@
       <c r="F153" s="4"/>
       <c r="G153" s="12"/>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A154" s="59"/>
       <c r="B154" s="57" t="s">
         <v>282</v>
@@ -11163,7 +11167,7 @@
       <c r="F154" s="4"/>
       <c r="G154" s="12"/>
     </row>
-    <row r="155" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A155" s="59"/>
       <c r="B155" s="34" t="s">
         <v>111</v>
@@ -11174,7 +11178,7 @@
       <c r="F155" s="42"/>
       <c r="G155" s="12"/>
     </row>
-    <row r="156" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A156" s="59"/>
       <c r="B156" s="57" t="s">
         <v>283</v>
@@ -11191,7 +11195,7 @@
       <c r="F156" s="4"/>
       <c r="G156" s="12"/>
     </row>
-    <row r="157" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A157" s="59"/>
       <c r="B157" s="34" t="s">
         <v>112</v>
@@ -11202,7 +11206,7 @@
       <c r="F157" s="42"/>
       <c r="G157" s="12"/>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A158" s="59"/>
       <c r="B158" s="57" t="s">
         <v>284</v>
@@ -11219,7 +11223,7 @@
       <c r="F158" s="4"/>
       <c r="G158" s="12"/>
     </row>
-    <row r="159" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A159" s="59"/>
       <c r="B159" s="34" t="s">
         <v>113</v>
@@ -11230,7 +11234,7 @@
       <c r="F159" s="42"/>
       <c r="G159" s="12"/>
     </row>
-    <row r="160" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A160" s="59"/>
       <c r="B160" s="57" t="s">
         <v>285</v>
@@ -11247,7 +11251,7 @@
       <c r="F160" s="4"/>
       <c r="G160" s="12"/>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A161" s="59"/>
       <c r="B161" s="57" t="s">
         <v>286</v>
@@ -11264,7 +11268,7 @@
       <c r="F161" s="4"/>
       <c r="G161" s="12"/>
     </row>
-    <row r="162" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A162" s="59"/>
       <c r="B162" s="57" t="s">
         <v>287</v>
@@ -11281,7 +11285,7 @@
       <c r="F162" s="4"/>
       <c r="G162" s="12"/>
     </row>
-    <row r="163" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A163" s="59"/>
       <c r="B163" s="34" t="s">
         <v>114</v>
@@ -11292,7 +11296,7 @@
       <c r="F163" s="42"/>
       <c r="G163" s="12"/>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A164" s="59"/>
       <c r="B164" s="57" t="s">
         <v>288</v>
@@ -11309,7 +11313,7 @@
       <c r="F164" s="4"/>
       <c r="G164" s="12"/>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A165" s="59"/>
       <c r="B165" s="57" t="s">
         <v>289</v>
@@ -11326,7 +11330,7 @@
       <c r="F165" s="4"/>
       <c r="G165" s="12"/>
     </row>
-    <row r="166" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A166" s="59"/>
       <c r="B166" s="57" t="s">
         <v>290</v>
@@ -11343,7 +11347,7 @@
       <c r="F166" s="4"/>
       <c r="G166" s="12"/>
     </row>
-    <row r="167" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A167" s="59"/>
       <c r="B167" s="57" t="s">
         <v>291</v>
@@ -11360,7 +11364,7 @@
       <c r="F167" s="4"/>
       <c r="G167" s="12"/>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A168" s="59"/>
       <c r="B168" s="57" t="s">
         <v>292</v>
@@ -11377,7 +11381,7 @@
       <c r="F168" s="4"/>
       <c r="G168" s="12"/>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A169" s="59"/>
       <c r="B169" s="57" t="s">
         <v>293</v>
@@ -11394,7 +11398,7 @@
       <c r="F169" s="4"/>
       <c r="G169" s="12"/>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A170" s="59"/>
       <c r="B170" s="69" t="s">
         <v>294</v>
@@ -11411,7 +11415,7 @@
       <c r="F170" s="70"/>
       <c r="G170" s="12"/>
     </row>
-    <row r="171" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A171" s="59"/>
       <c r="B171" s="34" t="s">
         <v>115</v>
@@ -11422,7 +11426,7 @@
       <c r="F171" s="42"/>
       <c r="G171" s="12"/>
     </row>
-    <row r="172" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A172" s="59"/>
       <c r="B172" s="57" t="s">
         <v>295</v>
@@ -11439,7 +11443,7 @@
       <c r="F172" s="4"/>
       <c r="G172" s="12"/>
     </row>
-    <row r="173" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A173" s="60"/>
       <c r="B173" s="58" t="s">
         <v>326</v>
@@ -11456,7 +11460,7 @@
       <c r="F173" s="44"/>
       <c r="G173" s="12"/>
     </row>
-    <row r="174" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" ht="53.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A174" s="59" t="s">
         <v>15</v>
       </c>
@@ -11469,7 +11473,7 @@
       <c r="F174" s="48"/>
       <c r="G174" s="12"/>
     </row>
-    <row r="175" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A175" s="59"/>
       <c r="B175" s="57" t="s">
         <v>296</v>
@@ -11486,7 +11490,7 @@
       <c r="F175" s="4"/>
       <c r="G175" s="12"/>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A176" s="59"/>
       <c r="B176" s="57" t="s">
         <v>297</v>
@@ -11503,7 +11507,7 @@
       <c r="F176" s="4"/>
       <c r="G176" s="12"/>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A177" s="59"/>
       <c r="B177" s="57" t="s">
         <v>298</v>
@@ -11520,7 +11524,7 @@
       <c r="F177" s="4"/>
       <c r="G177" s="12"/>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A178" s="59"/>
       <c r="B178" s="57" t="s">
         <v>299</v>
@@ -11537,7 +11541,7 @@
       <c r="F178" s="4"/>
       <c r="G178" s="12"/>
     </row>
-    <row r="179" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" ht="31.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A179" s="59"/>
       <c r="B179" s="57" t="s">
         <v>300</v>
@@ -11554,7 +11558,7 @@
       <c r="F179" s="4"/>
       <c r="G179" s="12"/>
     </row>
-    <row r="180" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A180" s="59"/>
       <c r="B180" s="34" t="s">
         <v>16</v>
@@ -11565,7 +11569,7 @@
       <c r="F180" s="42"/>
       <c r="G180" s="12"/>
     </row>
-    <row r="181" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" ht="46.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A181" s="59"/>
       <c r="B181" s="57" t="s">
         <v>301</v>
@@ -11582,7 +11586,7 @@
       <c r="F181" s="4"/>
       <c r="G181" s="12"/>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A182" s="59"/>
       <c r="B182" s="57" t="s">
         <v>302</v>
@@ -11599,7 +11603,7 @@
       <c r="F182" s="4"/>
       <c r="G182" s="12"/>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A183" s="59"/>
       <c r="B183" s="57" t="s">
         <v>303</v>
@@ -11616,7 +11620,7 @@
       <c r="F183" s="4"/>
       <c r="G183" s="12"/>
     </row>
-    <row r="184" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A184" s="59"/>
       <c r="B184" s="57" t="s">
         <v>304</v>
@@ -11633,7 +11637,7 @@
       <c r="F184" s="4"/>
       <c r="G184" s="12"/>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A185" s="59"/>
       <c r="B185" s="57" t="s">
         <v>305</v>
@@ -11650,7 +11654,7 @@
       <c r="F185" s="4"/>
       <c r="G185" s="12"/>
     </row>
-    <row r="186" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A186" s="59"/>
       <c r="B186" s="57" t="s">
         <v>306</v>
@@ -11667,7 +11671,7 @@
       <c r="F186" s="4"/>
       <c r="G186" s="12"/>
     </row>
-    <row r="187" spans="1:7" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" ht="93.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A187" s="59"/>
       <c r="B187" s="57" t="s">
         <v>307</v>
@@ -11684,7 +11688,7 @@
       <c r="F187" s="4"/>
       <c r="G187" s="12"/>
     </row>
-    <row r="188" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A188" s="59"/>
       <c r="B188" s="34" t="s">
         <v>117</v>
@@ -11695,7 +11699,7 @@
       <c r="F188" s="42"/>
       <c r="G188" s="12"/>
     </row>
-    <row r="189" spans="1:7" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:7" ht="47.1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A189" s="60"/>
       <c r="B189" s="58" t="s">
         <v>308</v>
@@ -11712,7 +11716,7 @@
       <c r="F189" s="44"/>
       <c r="G189" s="12"/>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A190" s="19" t="s">
         <v>17</v>
       </c>
@@ -11731,915 +11735,915 @@
       <c r="F190" s="41"/>
       <c r="G190" s="12"/>
     </row>
-    <row r="191" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A191" s="11"/>
       <c r="E191" s="28"/>
     </row>
-    <row r="192" spans="1:7" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A192" s="11"/>
       <c r="E192" s="28"/>
     </row>
-    <row r="193" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A193" s="11"/>
       <c r="E193" s="28"/>
     </row>
-    <row r="194" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A194" s="11"/>
       <c r="E194" s="28"/>
     </row>
-    <row r="195" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A195" s="11"/>
       <c r="E195" s="28"/>
     </row>
-    <row r="196" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A196" s="11"/>
       <c r="E196" s="28"/>
     </row>
-    <row r="197" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A197" s="11"/>
       <c r="E197" s="28"/>
     </row>
-    <row r="198" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A198" s="11"/>
       <c r="E198" s="28"/>
     </row>
-    <row r="199" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A199" s="11"/>
       <c r="E199" s="28"/>
     </row>
-    <row r="200" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A200" s="11"/>
       <c r="E200" s="28"/>
     </row>
-    <row r="201" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A201" s="11"/>
       <c r="E201" s="28"/>
     </row>
-    <row r="202" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A202" s="11"/>
       <c r="E202" s="28"/>
     </row>
-    <row r="203" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A203" s="11"/>
       <c r="E203" s="28"/>
     </row>
-    <row r="204" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A204" s="11"/>
       <c r="E204" s="28"/>
     </row>
-    <row r="205" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A205" s="11"/>
       <c r="E205" s="28"/>
     </row>
-    <row r="206" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A206" s="11"/>
       <c r="E206" s="28"/>
     </row>
-    <row r="207" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A207" s="11"/>
       <c r="E207" s="28"/>
     </row>
-    <row r="208" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A208" s="11"/>
       <c r="E208" s="28"/>
     </row>
-    <row r="209" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A209" s="11"/>
       <c r="E209" s="28"/>
     </row>
-    <row r="210" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A210" s="11"/>
       <c r="E210" s="28"/>
     </row>
-    <row r="211" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A211" s="11"/>
       <c r="E211" s="28"/>
     </row>
-    <row r="212" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A212" s="11"/>
       <c r="E212" s="28"/>
     </row>
-    <row r="213" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A213" s="11"/>
       <c r="E213" s="28"/>
     </row>
-    <row r="214" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A214" s="11"/>
       <c r="E214" s="28"/>
     </row>
-    <row r="215" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A215" s="11"/>
       <c r="E215" s="28"/>
     </row>
-    <row r="216" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A216" s="11"/>
       <c r="E216" s="28"/>
     </row>
-    <row r="217" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A217" s="11"/>
       <c r="E217" s="28"/>
     </row>
-    <row r="218" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A218" s="11"/>
       <c r="E218" s="28"/>
     </row>
-    <row r="219" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A219" s="11"/>
       <c r="E219" s="28"/>
     </row>
-    <row r="220" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A220" s="11"/>
       <c r="E220" s="28"/>
     </row>
-    <row r="221" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A221" s="11"/>
       <c r="E221" s="28"/>
     </row>
-    <row r="222" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A222" s="11"/>
       <c r="E222" s="28"/>
     </row>
-    <row r="223" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A223" s="11"/>
       <c r="E223" s="28"/>
     </row>
-    <row r="224" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A224" s="11"/>
       <c r="E224" s="28"/>
     </row>
-    <row r="225" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A225" s="11"/>
       <c r="E225" s="28"/>
     </row>
-    <row r="226" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A226" s="11"/>
       <c r="E226" s="28"/>
     </row>
-    <row r="227" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A227" s="11"/>
       <c r="E227" s="28"/>
     </row>
-    <row r="228" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A228" s="11"/>
       <c r="E228" s="28"/>
     </row>
-    <row r="229" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A229" s="11"/>
       <c r="E229" s="28"/>
     </row>
-    <row r="230" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A230" s="11"/>
       <c r="E230" s="28"/>
     </row>
-    <row r="231" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A231" s="11"/>
       <c r="E231" s="28"/>
     </row>
-    <row r="232" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A232" s="11"/>
       <c r="E232" s="28"/>
     </row>
-    <row r="233" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A233" s="11"/>
       <c r="E233" s="28"/>
     </row>
-    <row r="234" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A234" s="11"/>
       <c r="E234" s="28"/>
     </row>
-    <row r="235" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A235" s="11"/>
       <c r="E235" s="28"/>
     </row>
-    <row r="236" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A236" s="11"/>
       <c r="E236" s="28"/>
     </row>
-    <row r="237" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A237" s="11"/>
       <c r="E237" s="28"/>
     </row>
-    <row r="238" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A238" s="11"/>
       <c r="E238" s="28"/>
     </row>
-    <row r="239" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A239" s="11"/>
       <c r="E239" s="28"/>
     </row>
-    <row r="240" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A240" s="11"/>
       <c r="E240" s="28"/>
     </row>
-    <row r="241" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A241" s="11"/>
       <c r="E241" s="28"/>
     </row>
-    <row r="242" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A242" s="11"/>
       <c r="E242" s="28"/>
     </row>
-    <row r="243" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A243" s="11"/>
       <c r="E243" s="28"/>
     </row>
-    <row r="244" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A244" s="11"/>
       <c r="E244" s="28"/>
     </row>
-    <row r="245" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A245" s="11"/>
       <c r="E245" s="28"/>
     </row>
-    <row r="246" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A246" s="11"/>
       <c r="E246" s="28"/>
     </row>
-    <row r="247" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A247" s="11"/>
       <c r="E247" s="28"/>
     </row>
-    <row r="248" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A248" s="11"/>
       <c r="E248" s="28"/>
     </row>
-    <row r="249" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A249" s="11"/>
       <c r="E249" s="28"/>
     </row>
-    <row r="250" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A250" s="11"/>
       <c r="E250" s="28"/>
     </row>
-    <row r="251" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A251" s="11"/>
       <c r="E251" s="28"/>
     </row>
-    <row r="252" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A252" s="11"/>
       <c r="E252" s="28"/>
     </row>
-    <row r="253" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A253" s="11"/>
       <c r="E253" s="28"/>
     </row>
-    <row r="254" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A254" s="11"/>
       <c r="E254" s="28"/>
     </row>
-    <row r="255" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A255" s="11"/>
       <c r="E255" s="28"/>
     </row>
-    <row r="256" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A256" s="11"/>
       <c r="E256" s="28"/>
     </row>
-    <row r="257" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A257" s="11"/>
       <c r="E257" s="28"/>
     </row>
-    <row r="258" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A258" s="11"/>
       <c r="E258" s="28"/>
     </row>
-    <row r="259" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A259" s="11"/>
       <c r="E259" s="28"/>
     </row>
-    <row r="260" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A260" s="11"/>
       <c r="E260" s="28"/>
     </row>
-    <row r="261" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A261" s="11"/>
       <c r="E261" s="28"/>
     </row>
-    <row r="262" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A262" s="11"/>
       <c r="E262" s="28"/>
     </row>
-    <row r="263" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A263" s="11"/>
       <c r="E263" s="28"/>
     </row>
-    <row r="264" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A264" s="11"/>
       <c r="E264" s="28"/>
     </row>
-    <row r="265" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A265" s="11"/>
       <c r="E265" s="28"/>
     </row>
-    <row r="266" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A266" s="11"/>
       <c r="E266" s="28"/>
     </row>
-    <row r="267" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A267" s="11"/>
       <c r="E267" s="28"/>
     </row>
-    <row r="268" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A268" s="11"/>
       <c r="E268" s="28"/>
     </row>
-    <row r="269" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A269" s="11"/>
       <c r="E269" s="28"/>
     </row>
-    <row r="270" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A270" s="11"/>
       <c r="E270" s="28"/>
     </row>
-    <row r="271" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A271" s="11"/>
       <c r="E271" s="28"/>
     </row>
-    <row r="272" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A272" s="11"/>
       <c r="E272" s="28"/>
     </row>
-    <row r="273" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A273" s="11"/>
       <c r="E273" s="28"/>
     </row>
-    <row r="274" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A274" s="11"/>
       <c r="E274" s="28"/>
     </row>
-    <row r="275" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A275" s="11"/>
       <c r="E275" s="28"/>
     </row>
-    <row r="276" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A276" s="11"/>
       <c r="E276" s="28"/>
     </row>
-    <row r="277" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A277" s="11"/>
       <c r="E277" s="28"/>
     </row>
-    <row r="278" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A278" s="11"/>
       <c r="E278" s="28"/>
     </row>
-    <row r="279" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A279" s="11"/>
       <c r="E279" s="28"/>
     </row>
-    <row r="280" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A280" s="11"/>
       <c r="E280" s="28"/>
     </row>
-    <row r="281" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A281" s="11"/>
       <c r="E281" s="28"/>
     </row>
-    <row r="282" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A282" s="11"/>
       <c r="E282" s="28"/>
     </row>
-    <row r="283" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A283" s="11"/>
       <c r="E283" s="28"/>
     </row>
-    <row r="284" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A284" s="11"/>
       <c r="E284" s="28"/>
     </row>
-    <row r="285" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A285" s="11"/>
       <c r="E285" s="28"/>
     </row>
-    <row r="286" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A286" s="11"/>
       <c r="E286" s="28"/>
     </row>
-    <row r="287" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A287" s="11"/>
       <c r="E287" s="28"/>
     </row>
-    <row r="288" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A288" s="11"/>
       <c r="E288" s="28"/>
     </row>
-    <row r="289" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A289" s="11"/>
       <c r="E289" s="28"/>
     </row>
-    <row r="290" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A290" s="11"/>
       <c r="E290" s="28"/>
     </row>
-    <row r="291" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A291" s="11"/>
       <c r="E291" s="28"/>
     </row>
-    <row r="292" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A292" s="11"/>
       <c r="E292" s="28"/>
     </row>
-    <row r="293" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A293" s="11"/>
       <c r="E293" s="28"/>
     </row>
-    <row r="294" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A294" s="11"/>
       <c r="E294" s="28"/>
     </row>
-    <row r="295" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A295" s="11"/>
       <c r="E295" s="28"/>
     </row>
-    <row r="296" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A296" s="11"/>
       <c r="E296" s="28"/>
     </row>
-    <row r="297" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A297" s="11"/>
       <c r="E297" s="28"/>
     </row>
-    <row r="298" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A298" s="11"/>
       <c r="E298" s="28"/>
     </row>
-    <row r="299" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A299" s="11"/>
       <c r="E299" s="28"/>
     </row>
-    <row r="300" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A300" s="11"/>
       <c r="E300" s="28"/>
     </row>
-    <row r="301" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A301" s="11"/>
       <c r="E301" s="28"/>
     </row>
-    <row r="302" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A302" s="11"/>
       <c r="E302" s="28"/>
     </row>
-    <row r="303" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A303" s="11"/>
       <c r="E303" s="28"/>
     </row>
-    <row r="304" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A304" s="11"/>
       <c r="E304" s="28"/>
     </row>
-    <row r="305" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A305" s="11"/>
       <c r="E305" s="28"/>
     </row>
-    <row r="306" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A306" s="11"/>
       <c r="E306" s="28"/>
     </row>
-    <row r="307" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A307" s="11"/>
       <c r="E307" s="28"/>
     </row>
-    <row r="308" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A308" s="11"/>
       <c r="E308" s="28"/>
     </row>
-    <row r="309" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A309" s="11"/>
       <c r="E309" s="28"/>
     </row>
-    <row r="310" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A310" s="11"/>
       <c r="E310" s="28"/>
     </row>
-    <row r="311" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A311" s="11"/>
       <c r="E311" s="28"/>
     </row>
-    <row r="312" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A312" s="11"/>
       <c r="E312" s="28"/>
     </row>
-    <row r="313" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A313" s="11"/>
       <c r="E313" s="28"/>
     </row>
-    <row r="314" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A314" s="11"/>
       <c r="E314" s="28"/>
     </row>
-    <row r="315" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A315" s="11"/>
       <c r="E315" s="28"/>
     </row>
-    <row r="316" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A316" s="11"/>
       <c r="E316" s="28"/>
     </row>
-    <row r="317" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A317" s="11"/>
       <c r="E317" s="28"/>
     </row>
-    <row r="318" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A318" s="11"/>
       <c r="E318" s="28"/>
     </row>
-    <row r="319" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A319" s="11"/>
       <c r="E319" s="28"/>
     </row>
-    <row r="320" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A320" s="11"/>
       <c r="E320" s="28"/>
     </row>
-    <row r="321" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A321" s="11"/>
       <c r="E321" s="28"/>
     </row>
-    <row r="322" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A322" s="11"/>
       <c r="E322" s="28"/>
     </row>
-    <row r="323" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A323" s="11"/>
       <c r="E323" s="28"/>
     </row>
-    <row r="324" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A324" s="11"/>
       <c r="E324" s="28"/>
     </row>
-    <row r="325" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A325" s="11"/>
       <c r="E325" s="28"/>
     </row>
-    <row r="326" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A326" s="11"/>
       <c r="E326" s="28"/>
     </row>
-    <row r="327" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A327" s="11"/>
       <c r="E327" s="28"/>
     </row>
-    <row r="328" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A328" s="11"/>
       <c r="E328" s="28"/>
     </row>
-    <row r="329" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A329" s="11"/>
       <c r="E329" s="28"/>
     </row>
-    <row r="330" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A330" s="11"/>
       <c r="E330" s="28"/>
     </row>
-    <row r="331" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A331" s="11"/>
       <c r="E331" s="28"/>
     </row>
-    <row r="332" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A332" s="11"/>
       <c r="E332" s="28"/>
     </row>
-    <row r="333" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A333" s="11"/>
       <c r="E333" s="28"/>
     </row>
-    <row r="334" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A334" s="11"/>
       <c r="E334" s="28"/>
     </row>
-    <row r="335" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A335" s="11"/>
       <c r="E335" s="28"/>
     </row>
-    <row r="336" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A336" s="11"/>
       <c r="E336" s="28"/>
     </row>
-    <row r="337" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A337" s="11"/>
       <c r="E337" s="28"/>
     </row>
-    <row r="338" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A338" s="11"/>
       <c r="E338" s="28"/>
     </row>
-    <row r="339" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A339" s="11"/>
       <c r="E339" s="28"/>
     </row>
-    <row r="340" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A340" s="11"/>
       <c r="E340" s="28"/>
     </row>
-    <row r="341" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A341" s="11"/>
       <c r="E341" s="28"/>
     </row>
-    <row r="342" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A342" s="11"/>
       <c r="E342" s="28"/>
     </row>
-    <row r="343" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A343" s="11"/>
       <c r="E343" s="28"/>
     </row>
-    <row r="344" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A344" s="11"/>
       <c r="E344" s="28"/>
     </row>
-    <row r="345" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A345" s="11"/>
       <c r="E345" s="28"/>
     </row>
-    <row r="346" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A346" s="11"/>
       <c r="E346" s="28"/>
     </row>
-    <row r="347" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A347" s="11"/>
       <c r="E347" s="28"/>
     </row>
-    <row r="348" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A348" s="11"/>
       <c r="E348" s="28"/>
     </row>
-    <row r="349" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A349" s="11"/>
       <c r="E349" s="28"/>
     </row>
-    <row r="350" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A350" s="11"/>
       <c r="E350" s="28"/>
     </row>
-    <row r="351" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A351" s="11"/>
       <c r="E351" s="28"/>
     </row>
-    <row r="352" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A352" s="11"/>
       <c r="E352" s="28"/>
     </row>
-    <row r="353" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A353" s="11"/>
       <c r="E353" s="28"/>
     </row>
-    <row r="354" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A354" s="11"/>
       <c r="E354" s="28"/>
     </row>
-    <row r="355" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A355" s="11"/>
       <c r="E355" s="28"/>
     </row>
-    <row r="356" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A356" s="11"/>
       <c r="E356" s="28"/>
     </row>
-    <row r="357" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A357" s="11"/>
       <c r="E357" s="28"/>
     </row>
-    <row r="358" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A358" s="11"/>
       <c r="E358" s="28"/>
     </row>
-    <row r="359" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A359" s="11"/>
       <c r="E359" s="28"/>
     </row>
-    <row r="360" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A360" s="11"/>
       <c r="E360" s="28"/>
     </row>
-    <row r="361" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A361" s="11"/>
       <c r="E361" s="28"/>
     </row>
-    <row r="362" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A362" s="11"/>
       <c r="E362" s="28"/>
     </row>
-    <row r="363" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A363" s="11"/>
       <c r="E363" s="28"/>
     </row>
-    <row r="364" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A364" s="11"/>
       <c r="E364" s="28"/>
     </row>
-    <row r="365" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A365" s="11"/>
       <c r="E365" s="28"/>
     </row>
-    <row r="366" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A366" s="11"/>
       <c r="E366" s="28"/>
     </row>
-    <row r="367" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A367" s="11"/>
       <c r="E367" s="28"/>
     </row>
-    <row r="368" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A368" s="11"/>
       <c r="E368" s="28"/>
     </row>
-    <row r="369" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A369" s="11"/>
       <c r="E369" s="28"/>
     </row>
-    <row r="370" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A370" s="11"/>
       <c r="E370" s="28"/>
     </row>
-    <row r="371" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A371" s="11"/>
       <c r="E371" s="28"/>
     </row>
-    <row r="372" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A372" s="11"/>
       <c r="E372" s="28"/>
     </row>
-    <row r="373" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A373" s="11"/>
       <c r="E373" s="28"/>
     </row>
-    <row r="374" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A374" s="11"/>
       <c r="E374" s="28"/>
     </row>
-    <row r="375" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A375" s="11"/>
       <c r="E375" s="28"/>
     </row>
-    <row r="376" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A376" s="11"/>
       <c r="E376" s="28"/>
     </row>
-    <row r="377" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A377" s="11"/>
       <c r="E377" s="28"/>
     </row>
-    <row r="378" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A378" s="11"/>
       <c r="E378" s="28"/>
     </row>
-    <row r="379" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A379" s="11"/>
       <c r="E379" s="28"/>
     </row>
-    <row r="380" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A380" s="11"/>
       <c r="E380" s="28"/>
     </row>
-    <row r="381" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A381" s="11"/>
       <c r="E381" s="28"/>
     </row>
-    <row r="382" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A382" s="11"/>
       <c r="E382" s="28"/>
     </row>
-    <row r="383" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A383" s="11"/>
       <c r="E383" s="28"/>
     </row>
-    <row r="384" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A384" s="11"/>
       <c r="E384" s="28"/>
     </row>
-    <row r="385" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A385" s="11"/>
       <c r="E385" s="28"/>
     </row>
-    <row r="386" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A386" s="11"/>
       <c r="E386" s="28"/>
     </row>
-    <row r="387" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A387" s="11"/>
       <c r="E387" s="28"/>
     </row>
-    <row r="388" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A388" s="11"/>
       <c r="E388" s="28"/>
     </row>
-    <row r="389" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A389" s="11"/>
       <c r="E389" s="28"/>
     </row>
-    <row r="390" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A390" s="11"/>
       <c r="E390" s="28"/>
     </row>
-    <row r="391" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A391" s="11"/>
       <c r="E391" s="28"/>
     </row>
-    <row r="392" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A392" s="11"/>
       <c r="E392" s="28"/>
     </row>
-    <row r="393" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A393" s="11"/>
       <c r="E393" s="28"/>
     </row>
-    <row r="394" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A394" s="11"/>
       <c r="E394" s="28"/>
     </row>
-    <row r="395" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A395" s="11"/>
       <c r="E395" s="28"/>
     </row>
-    <row r="396" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A396" s="11"/>
       <c r="E396" s="28"/>
     </row>
-    <row r="397" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A397" s="11"/>
       <c r="E397" s="28"/>
     </row>
-    <row r="398" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A398" s="11"/>
       <c r="E398" s="28"/>
     </row>
-    <row r="399" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A399" s="11"/>
       <c r="E399" s="28"/>
     </row>
-    <row r="400" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A400" s="11"/>
       <c r="E400" s="28"/>
     </row>
-    <row r="401" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A401" s="11"/>
       <c r="E401" s="28"/>
     </row>
-    <row r="402" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A402" s="11"/>
       <c r="E402" s="28"/>
     </row>
-    <row r="403" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A403" s="11"/>
       <c r="E403" s="28"/>
     </row>
-    <row r="404" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A404" s="11"/>
       <c r="E404" s="28"/>
     </row>
-    <row r="405" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A405" s="11"/>
       <c r="E405" s="28"/>
     </row>
-    <row r="406" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A406" s="11"/>
       <c r="E406" s="28"/>
     </row>
-    <row r="407" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A407" s="11"/>
       <c r="E407" s="28"/>
     </row>
-    <row r="408" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A408" s="11"/>
       <c r="E408" s="28"/>
     </row>
-    <row r="409" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A409" s="11"/>
       <c r="E409" s="28"/>
     </row>
-    <row r="410" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A410" s="11"/>
       <c r="E410" s="28"/>
     </row>
-    <row r="411" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A411" s="11"/>
       <c r="E411" s="28"/>
     </row>
-    <row r="412" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A412" s="11"/>
       <c r="E412" s="28"/>
     </row>
-    <row r="413" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A413" s="11"/>
       <c r="E413" s="28"/>
     </row>
-    <row r="414" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A414" s="11"/>
       <c r="E414" s="28"/>
     </row>
-    <row r="415" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A415" s="11"/>
       <c r="E415" s="28"/>
     </row>
-    <row r="416" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A416" s="11"/>
       <c r="E416" s="28"/>
     </row>
-    <row r="417" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A417" s="11"/>
       <c r="E417" s="28"/>
     </row>
-    <row r="418" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:5" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A418" s="11"/>
       <c r="E418" s="28"/>
     </row>
@@ -12712,38 +12716,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <g8cc7f6e98b34d1387cc1791a9d2d9a3 xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </g8cc7f6e98b34d1387cc1791a9d2d9a3>
-    <MSB_RecordId xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f" xsi:nil="true"/>
-    <l327da1f1d44497ab3337057f4d04951 xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Standard</TermName>
-          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">42db7290-f92b-446b-999c-1bee6d848af0</TermId>
-        </TermInfo>
-      </Terms>
-    </l327da1f1d44497ab3337057f4d04951>
-    <msbLabel xmlns="09080109-f6cd-4eba-a2ee-73217fe696ed"/>
-    <TaxCatchAll xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f">
-      <Value>1</Value>
-    </TaxCatchAll>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="MSB Dokument" ma:contentTypeID="0x0101008239AB5D3D2647B580F011DA2F35611101000A86203C37271B42A7865B88E83F44AE" ma:contentTypeVersion="6" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="e9dd56b95f539d61232eda99a945ba42">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="09080109-f6cd-4eba-a2ee-73217fe696ed" xmlns:ns3="06622f86-497a-49b5-9d4e-f3ea00047d2f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="face33d3ab82312ff826d0b7d541885e" ns2:_="" ns3:_="">
     <xsd:import namespace="09080109-f6cd-4eba-a2ee-73217fe696ed"/>
@@ -12954,10 +12926,53 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <g8cc7f6e98b34d1387cc1791a9d2d9a3 xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </g8cc7f6e98b34d1387cc1791a9d2d9a3>
+    <MSB_RecordId xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f" xsi:nil="true"/>
+    <l327da1f1d44497ab3337057f4d04951 xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+        <TermInfo xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+          <TermName xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">Standard</TermName>
+          <TermId xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">42db7290-f92b-446b-999c-1bee6d848af0</TermId>
+        </TermInfo>
+      </Terms>
+    </l327da1f1d44497ab3337057f4d04951>
+    <msbLabel xmlns="09080109-f6cd-4eba-a2ee-73217fe696ed"/>
+    <TaxCatchAll xmlns="06622f86-497a-49b5-9d4e-f3ea00047d2f">
+      <Value>1</Value>
+    </TaxCatchAll>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74E39A40-EF53-41B0-AE0C-BDF1760CF50B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F79A66C0-FFFC-4B90-B71D-9721290EB3C8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="09080109-f6cd-4eba-a2ee-73217fe696ed"/>
+    <ds:schemaRef ds:uri="06622f86-497a-49b5-9d4e-f3ea00047d2f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -12980,20 +12995,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F79A66C0-FFFC-4B90-B71D-9721290EB3C8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74E39A40-EF53-41B0-AE0C-BDF1760CF50B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="09080109-f6cd-4eba-a2ee-73217fe696ed"/>
-    <ds:schemaRef ds:uri="06622f86-497a-49b5-9d4e-f3ea00047d2f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>